<commit_message>
Actually add the Send Resume column to the tracker
The previous commit claimed this and did not deliver it: the patch script hit a
failed no-op assertion and exited before writing tracker.py, so the column never
existed. Verified present this time, with the cell colour-coded blue for the
mobile resume and green for the MERN one, and "(check)" appended whenever the
router's confidence is below high.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/tracker.xlsx
+++ b/reports/tracker.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Founder Targets" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$P$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Listings'!$A$1:$Q$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,12 @@
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00197A55"/>
       <sz val="10"/>
     </font>
     <font>
@@ -63,7 +69,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -80,6 +86,11 @@
         <fgColor rgb="00E3F1EA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D8EEE2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -93,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -104,16 +115,19 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -479,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -493,11 +507,12 @@
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="52" customWidth="1" min="13" max="13"/>
-    <col width="60" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="58" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="38" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -558,25 +573,30 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Send Resume</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Apply</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>JD Link</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Tailor Command</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Applied?</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -626,21 +646,26 @@
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
+          <t>MERN (check)</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="N2" s="6" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/gohighlevel/13c8402f-8cf0-4b09-b666-43e71b8b525e</t>
         </is>
       </c>
-      <c r="N2" s="6" t="inlineStr">
+      <c r="O2" s="7" t="inlineStr">
         <is>
           <t>node scripts/tailor.mjs --url "https://jobs.lever.co/gohighlevel/13c8402f-8cf0-4b09-b666-43e71b8b525e" --company "HighLevel (GoHighLevel)" --title "Software Development Engineer II - Backend"</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>On-site or hybrid at a named Indian location.</t>
         </is>
@@ -690,21 +715,26 @@
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
+          <t>MERN (check)</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/gohighlevel/b8dc97ec-a0b7-4195-9f3b-86440ff18f82</t>
         </is>
       </c>
-      <c r="N3" s="6" t="inlineStr">
+      <c r="O3" s="7" t="inlineStr">
         <is>
           <t>node scripts/tailor.mjs --url "https://jobs.lever.co/gohighlevel/b8dc97ec-a0b7-4195-9f3b-86440ff18f82" --company "HighLevel (GoHighLevel)" --title "Software Development Engineer II - Frontend"</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>On-site or hybrid at a named Indian location.</t>
         </is>
@@ -754,21 +784,26 @@
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
+          <t>MERN (check)</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>https://apply.workable.com/j/E7CD7FB957</t>
         </is>
       </c>
-      <c r="N4" s="6" t="inlineStr">
+      <c r="O4" s="7" t="inlineStr">
         <is>
           <t>node scripts/tailor.mjs --url "https://apply.workable.com/j/E7CD7FB957" --company "Innovaccer" --title "4403 - Software Development Engineer-II (Finance - AI Engineering)"</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>On-site or hybrid at a named Indian location. | Weak archetype match (best: sde-generalist @ 16)</t>
         </is>
@@ -818,21 +853,26 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
+          <t>MERN</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/gitlab/jobs/8775507002</t>
         </is>
       </c>
-      <c r="N5" s="6" t="inlineStr">
+      <c r="O5" s="7" t="inlineStr">
         <is>
           <t>node scripts/tailor.mjs --url "https://job-boards.greenhouse.io/gitlab/jobs/8775507002" --company "GitLab" --title "Intermediate Backend Engineer, India"</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="3" t="inlineStr">
         <is>
           <t>On-site or hybrid at a named Indian location.</t>
         </is>
@@ -882,21 +922,26 @@
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
+          <t>MERN</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/gitlab/jobs/8736877002</t>
         </is>
       </c>
-      <c r="N6" s="6" t="inlineStr">
+      <c r="O6" s="7" t="inlineStr">
         <is>
           <t>node scripts/tailor.mjs --url "https://job-boards.greenhouse.io/gitlab/jobs/8736877002" --company "GitLab" --title "Intermediate Backend Engineer"</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr"/>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="3" t="inlineStr">
         <is>
           <t>On-site or hybrid at a named Indian location.</t>
         </is>
@@ -950,21 +995,26 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
+          <t>MERN</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/supabase/06752423-eebb-472c-95b5-c7ff2559fd60</t>
         </is>
       </c>
-      <c r="N7" s="6" t="inlineStr">
+      <c r="O7" s="7" t="inlineStr">
         <is>
           <t>node scripts/tailor.mjs --url "https://jobs.ashbyhq.com/supabase/06752423-eebb-472c-95b5-c7ff2559fd60" --company "Supabase" --title "Software Engineer - Branching"</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr"/>
-      <c r="P7" s="3" t="inlineStr">
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="3" t="inlineStr">
         <is>
           <t>Worldwide or "anywhere" with no country lock stated.</t>
         </is>
@@ -1018,21 +1068,26 @@
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
+          <t>MERN</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="M8" s="5" t="inlineStr">
+      <c r="N8" s="6" t="inlineStr">
         <is>
           <t>https://apply.workable.com/j/6FB4B40CD6</t>
         </is>
       </c>
-      <c r="N8" s="6" t="inlineStr">
+      <c r="O8" s="7" t="inlineStr">
         <is>
           <t>node scripts/tailor.mjs --url "https://apply.workable.com/j/6FB4B40CD6" --company "Innovaccer" --title "4423- Software Development Engineer-II Backend"</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr"/>
-      <c r="P8" s="3" t="inlineStr">
+      <c r="P8" s="2" t="inlineStr"/>
+      <c r="Q8" s="3" t="inlineStr">
         <is>
           <t>On-site or hybrid at a named Indian location.</t>
         </is>
@@ -1082,21 +1137,26 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
+          <t>MERN</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="N9" s="6" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/gitlab/jobs/8722304002</t>
         </is>
       </c>
-      <c r="N9" s="6" t="inlineStr">
+      <c r="O9" s="7" t="inlineStr">
         <is>
           <t>node scripts/tailor.mjs --url "https://job-boards.greenhouse.io/gitlab/jobs/8722304002" --company "GitLab" --title "Intermediate Backend Engineer - Database Change Management"</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr"/>
-      <c r="P9" s="3" t="inlineStr">
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="3" t="inlineStr">
         <is>
           <t>On-site or hybrid at a named Indian location.</t>
         </is>
@@ -1150,21 +1210,26 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
+          <t>MERN</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="N10" s="6" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/aiprise/02112df8-70fa-4133-a860-151b5f585ed9</t>
         </is>
       </c>
-      <c r="N10" s="6" t="inlineStr">
+      <c r="O10" s="7" t="inlineStr">
         <is>
           <t>node scripts/tailor.mjs --url "https://jobs.ashbyhq.com/aiprise/02112df8-70fa-4133-a860-151b5f585ed9" --company "AiPrise" --title "Software Engineer II (Bangalore, India)"</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr"/>
-      <c r="P10" s="3" t="inlineStr">
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="3" t="inlineStr">
         <is>
           <t>On-site or hybrid at a named Indian location.</t>
         </is>
@@ -1214,21 +1279,26 @@
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
+          <t>MERN</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="N11" s="6" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/aiprise/3763c791-a387-4078-9ca4-00cbfbf9b1a6</t>
         </is>
       </c>
-      <c r="N11" s="6" t="inlineStr">
+      <c r="O11" s="7" t="inlineStr">
         <is>
           <t>node scripts/tailor.mjs --url "https://jobs.ashbyhq.com/aiprise/3763c791-a387-4078-9ca4-00cbfbf9b1a6" --company "AiPrise" --title "Software Engineer I (Bangalore, India)"</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr"/>
-      <c r="P11" s="3" t="inlineStr">
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="3" t="inlineStr">
         <is>
           <t>On-site or hybrid at a named Indian location.</t>
         </is>
@@ -1282,21 +1352,26 @@
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
+          <t>MERN</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="N12" s="6" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/aiprise/e7890d9f-8e1f-48a0-92be-071a282e7fe8</t>
         </is>
       </c>
-      <c r="N12" s="6" t="inlineStr">
+      <c r="O12" s="7" t="inlineStr">
         <is>
           <t>node scripts/tailor.mjs --url "https://jobs.ashbyhq.com/aiprise/e7890d9f-8e1f-48a0-92be-071a282e7fe8" --company "AiPrise" --title "Software Engineer III (Bangalore, India)"</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr"/>
-      <c r="P12" s="3" t="inlineStr">
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="3" t="inlineStr">
         <is>
           <t>On-site or hybrid at a named Indian location.</t>
         </is>
@@ -1350,21 +1425,26 @@
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
+          <t>MERN</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="N13" s="6" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/dscout/jobs/4370266009</t>
         </is>
       </c>
-      <c r="N13" s="6" t="inlineStr">
+      <c r="O13" s="7" t="inlineStr">
         <is>
           <t>node scripts/tailor.mjs --url "https://job-boards.greenhouse.io/dscout/jobs/4370266009" --company "Dscout" --title "Software Engineer - India"</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr"/>
-      <c r="P13" s="3" t="inlineStr">
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="3" t="inlineStr">
         <is>
           <t>Remote and India is named explicitly.</t>
         </is>
@@ -1414,55 +1494,60 @@
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
+          <t>MERN (check)</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="M14" s="5" t="inlineStr">
+      <c r="N14" s="6" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/gleanwork/jobs/4722386005</t>
         </is>
       </c>
-      <c r="N14" s="6" t="inlineStr">
+      <c r="O14" s="7" t="inlineStr">
         <is>
           <t>node scripts/tailor.mjs --url "https://job-boards.greenhouse.io/gleanwork/jobs/4722386005" --company "Glean" --title "Strategic Solutions Engineer, West"</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr"/>
-      <c r="P14" s="3" t="inlineStr">
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="3" t="inlineStr">
         <is>
           <t>Plain "Remote" with no country lock stated. Verify India eligibility on the JD before applying. | Negative keywords: servicenow</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P14"/>
+  <autoFilter ref="A1:Q14"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1578,7 +1663,7 @@
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>VERIFY BEFORE SENDING — every Guessed Email is a first@domain guess, never a verified address; check it yourself (Hunter.io) first. Personalise every draft with one genuine observation about what they build. Nothing in this tab is ever sent automatically.</t>
         </is>

</xml_diff>